<commit_message>
Continuing work working through output tables.
</commit_message>
<xml_diff>
--- a/output_tables/group_summary2.xlsx
+++ b/output_tables/group_summary2.xlsx
@@ -8,19 +8,36 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://stateofwa-my.sharepoint.com/personal/peter_dowty_dnr_wa_gov/Documents/projects/seagrass_restoration_data_2026/output_tables/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="12" documentId="8_{F177984F-47C9-4DF3-9790-FCF47BF4A52E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{94D2AB0F-17B2-4767-93A9-21E131BB17F4}"/>
+  <xr:revisionPtr revIDLastSave="59" documentId="8_{F177984F-47C9-4DF3-9790-FCF47BF4A52E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0C858AC5-6A0C-4B66-86AD-61A0C71D6E0A}"/>
   <bookViews>
-    <workbookView xWindow="165" yWindow="390" windowWidth="28635" windowHeight="15390" xr2:uid="{BE2CE89B-6CC7-4C87-B512-09CA381F0A6E}"/>
+    <workbookView xWindow="-15" yWindow="120" windowWidth="28635" windowHeight="15390" xr2:uid="{BE2CE89B-6CC7-4C87-B512-09CA381F0A6E}"/>
   </bookViews>
   <sheets>
     <sheet name="group_summary2" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">group_summary2!$E$1:$E$197</definedName>
+    <definedName name="_xlnm.Extract" localSheetId="0">group_summary2!$H$4</definedName>
+  </definedNames>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="592" uniqueCount="201">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="632" uniqueCount="210">
   <si>
     <t>group_no</t>
   </si>
@@ -623,13 +640,40 @@
   </si>
   <si>
     <t>ZAN_4</t>
+  </si>
+  <si>
+    <t>BESE case - needs to be addressed somehow</t>
+  </si>
+  <si>
+    <t>needs resolution - a 4-record polygon planting with different method for each corner; "drop"</t>
+  </si>
+  <si>
+    <t>needs resolution - a 4-record polygon planting with different method for each corner; "retain"</t>
+  </si>
+  <si>
+    <t>Is the 'mix' specifically drawn from the other test cases at BB_test_1?</t>
+  </si>
+  <si>
+    <t>List of unique donor sites</t>
+  </si>
+  <si>
+    <t>count</t>
+  </si>
+  <si>
+    <t>total n</t>
+  </si>
+  <si>
+    <t>n cases with multiple donor sites</t>
+  </si>
+  <si>
+    <t>BESE case - needs to be addressed somehow. Activity filter gives multiple BESE planting locations as one group, but these are distinct in location and coords</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -760,6 +804,13 @@
     <font>
       <sz val="11"/>
       <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="16"/>
+      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -958,7 +1009,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="11">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -1088,6 +1139,15 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -1133,10 +1193,13 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1193,6 +1256,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1512,7 +1579,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D0844630-C3CC-4326-9A50-3DDD6181A5BD}">
-  <dimension ref="A1:E197"/>
+  <dimension ref="A1:L197"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
@@ -1520,9 +1587,12 @@
     <col min="3" max="3" width="19" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="8.28515625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="29.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="144.42578125" customWidth="1"/>
+    <col min="7" max="7" width="15.140625" customWidth="1"/>
+    <col min="8" max="8" width="29.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1536,7 +1606,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" ht="21" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1552,8 +1622,11 @@
       <c r="E2" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H2" s="3" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1570,7 +1643,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1586,8 +1659,14 @@
       <c r="E4" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="I4" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1603,8 +1682,15 @@
       <c r="E5" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H5" t="s">
+        <v>26</v>
+      </c>
+      <c r="I5">
+        <f>COUNTIF(E:E,H5)</f>
+        <v>49</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1620,8 +1706,22 @@
       <c r="E6" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H6" t="s">
+        <v>16</v>
+      </c>
+      <c r="I6">
+        <f>COUNTIF(E:E,H6)</f>
+        <v>21</v>
+      </c>
+      <c r="K6">
+        <f>SUM(I5:I33)</f>
+        <v>196</v>
+      </c>
+      <c r="L6" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1637,8 +1737,22 @@
       <c r="E7" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H7" t="s">
+        <v>31</v>
+      </c>
+      <c r="I7">
+        <f>COUNTIF(E:E,H7)</f>
+        <v>20</v>
+      </c>
+      <c r="K7">
+        <f>SUM(I29:I33)</f>
+        <v>10</v>
+      </c>
+      <c r="L7" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1654,8 +1768,15 @@
       <c r="E8" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H8" t="s">
+        <v>6</v>
+      </c>
+      <c r="I8">
+        <f>COUNTIF(E:E,H8)</f>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1671,8 +1792,19 @@
       <c r="E9" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H9" t="s">
+        <v>60</v>
+      </c>
+      <c r="I9">
+        <f>COUNTIF(E:E,H9)</f>
+        <v>11</v>
+      </c>
+      <c r="K9" s="4">
+        <f>K7/K6</f>
+        <v>5.1020408163265307E-2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1688,8 +1820,15 @@
       <c r="E10" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H10" t="s">
+        <v>144</v>
+      </c>
+      <c r="I10">
+        <f>COUNTIF(E:E,H10)</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1705,8 +1844,15 @@
       <c r="E11" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H11" t="s">
+        <v>166</v>
+      </c>
+      <c r="I11">
+        <f>COUNTIF(E:E,H11)</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1722,8 +1868,15 @@
       <c r="E12" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H12" t="s">
+        <v>12</v>
+      </c>
+      <c r="I12">
+        <f>COUNTIF(E:E,H12)</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1739,8 +1892,15 @@
       <c r="E13" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H13" t="s">
+        <v>22</v>
+      </c>
+      <c r="I13">
+        <f>COUNTIF(E:E,H13)</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1756,8 +1916,15 @@
       <c r="E14" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H14" t="s">
+        <v>37</v>
+      </c>
+      <c r="I14">
+        <f>COUNTIF(E:E,H14)</f>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
@@ -1773,8 +1940,15 @@
       <c r="E15" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H15" t="s">
+        <v>45</v>
+      </c>
+      <c r="I15">
+        <f>COUNTIF(E:E,H15)</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>15</v>
       </c>
@@ -1790,8 +1964,15 @@
       <c r="E16" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H16" t="s">
+        <v>179</v>
+      </c>
+      <c r="I16">
+        <f>COUNTIF(E:E,H16)</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1807,8 +1988,15 @@
       <c r="E17" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H17" t="s">
+        <v>9</v>
+      </c>
+      <c r="I17">
+        <f>COUNTIF(E:E,H17)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>17</v>
       </c>
@@ -1824,8 +2012,15 @@
       <c r="E18" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H18" t="s">
+        <v>33</v>
+      </c>
+      <c r="I18">
+        <f>COUNTIF(E:E,H18)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>18</v>
       </c>
@@ -1841,8 +2036,15 @@
       <c r="E19" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H19" t="s">
+        <v>32</v>
+      </c>
+      <c r="I19">
+        <f>COUNTIF(E:E,H19)</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>19</v>
       </c>
@@ -1858,8 +2060,15 @@
       <c r="E20" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H20" t="s">
+        <v>34</v>
+      </c>
+      <c r="I20">
+        <f>COUNTIF(E:E,H20)</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>20</v>
       </c>
@@ -1875,8 +2084,15 @@
       <c r="E21" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H21" t="s">
+        <v>64</v>
+      </c>
+      <c r="I21">
+        <f>COUNTIF(E:E,H21)</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>21</v>
       </c>
@@ -1892,8 +2108,15 @@
       <c r="E22" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H22" t="s">
+        <v>120</v>
+      </c>
+      <c r="I22">
+        <f>COUNTIF(E:E,H22)</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>22</v>
       </c>
@@ -1909,8 +2132,18 @@
       <c r="E23" s="2" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F23" t="s">
+        <v>204</v>
+      </c>
+      <c r="H23" t="s">
+        <v>186</v>
+      </c>
+      <c r="I23">
+        <f>COUNTIF(E:E,H23)</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>23</v>
       </c>
@@ -1926,8 +2159,15 @@
       <c r="E24" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H24" t="s">
+        <v>52</v>
+      </c>
+      <c r="I24">
+        <f>COUNTIF(E:E,H24)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>24</v>
       </c>
@@ -1943,8 +2183,15 @@
       <c r="E25" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H25" t="s">
+        <v>76</v>
+      </c>
+      <c r="I25">
+        <f>COUNTIF(E:E,H25)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>25</v>
       </c>
@@ -1960,8 +2207,15 @@
       <c r="E26" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H26" t="s">
+        <v>177</v>
+      </c>
+      <c r="I26">
+        <f>COUNTIF(E:E,H26)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>26</v>
       </c>
@@ -1977,8 +2231,15 @@
       <c r="E27" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H27" t="s">
+        <v>191</v>
+      </c>
+      <c r="I27">
+        <f>COUNTIF(E:E,H27)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>27</v>
       </c>
@@ -1994,8 +2255,15 @@
       <c r="E28" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H28" s="5" t="s">
+        <v>193</v>
+      </c>
+      <c r="I28" s="5">
+        <f>COUNTIF(E:E,H28)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>28</v>
       </c>
@@ -2011,8 +2279,15 @@
       <c r="E29" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H29" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="I29">
+        <f t="shared" ref="I6:I33" si="0">COUNTIF(E:E,H29)</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>29</v>
       </c>
@@ -2028,8 +2303,15 @@
       <c r="E30" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H30" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="I30">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>30</v>
       </c>
@@ -2045,8 +2327,15 @@
       <c r="E31" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H31" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="I31">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>31</v>
       </c>
@@ -2062,8 +2351,15 @@
       <c r="E32" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H32" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="I32">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>32</v>
       </c>
@@ -2079,8 +2375,15 @@
       <c r="E33" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H33" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="I33">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>33</v>
       </c>
@@ -2097,7 +2400,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>34</v>
       </c>
@@ -2114,7 +2417,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>35</v>
       </c>
@@ -2131,7 +2434,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>36</v>
       </c>
@@ -2148,7 +2451,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>37</v>
       </c>
@@ -2165,7 +2468,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>38</v>
       </c>
@@ -2182,7 +2485,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>39</v>
       </c>
@@ -2199,7 +2502,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>40</v>
       </c>
@@ -2216,7 +2519,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>41</v>
       </c>
@@ -2233,7 +2536,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>42</v>
       </c>
@@ -2250,7 +2553,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>43</v>
       </c>
@@ -2267,7 +2570,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>44</v>
       </c>
@@ -2284,7 +2587,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>45</v>
       </c>
@@ -2301,7 +2604,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>46</v>
       </c>
@@ -2318,7 +2621,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>47</v>
       </c>
@@ -2879,7 +3182,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A81">
         <v>80</v>
       </c>
@@ -2896,7 +3199,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A82">
         <v>81</v>
       </c>
@@ -2913,7 +3216,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A83">
         <v>82</v>
       </c>
@@ -2930,7 +3233,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A84">
         <v>83</v>
       </c>
@@ -2947,7 +3250,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A85">
         <v>84</v>
       </c>
@@ -2964,7 +3267,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A86">
         <v>85</v>
       </c>
@@ -2981,7 +3284,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A87">
         <v>86</v>
       </c>
@@ -2998,7 +3301,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A88">
         <v>87</v>
       </c>
@@ -3015,7 +3318,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A89">
         <v>88</v>
       </c>
@@ -3031,8 +3334,11 @@
       <c r="E89" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F89" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A90">
         <v>89</v>
       </c>
@@ -3048,8 +3354,11 @@
       <c r="E90" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F90" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A91">
         <v>90</v>
       </c>
@@ -3065,8 +3374,11 @@
       <c r="E91" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F91" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A92">
         <v>91</v>
       </c>
@@ -3082,8 +3394,11 @@
       <c r="E92" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F92" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A93">
         <v>92</v>
       </c>
@@ -3100,7 +3415,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A94">
         <v>93</v>
       </c>
@@ -3117,7 +3432,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A95">
         <v>94</v>
       </c>
@@ -3134,7 +3449,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A96">
         <v>95</v>
       </c>
@@ -3151,7 +3466,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A97">
         <v>96</v>
       </c>
@@ -3167,8 +3482,11 @@
       <c r="E97" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F97" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A98">
         <v>97</v>
       </c>
@@ -3185,7 +3503,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A99">
         <v>98</v>
       </c>
@@ -3202,7 +3520,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A100">
         <v>99</v>
       </c>
@@ -3219,7 +3537,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A101">
         <v>100</v>
       </c>
@@ -3236,7 +3554,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A102">
         <v>101</v>
       </c>
@@ -3253,7 +3571,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A103">
         <v>102</v>
       </c>
@@ -3270,7 +3588,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A104">
         <v>103</v>
       </c>
@@ -3287,7 +3605,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A105">
         <v>104</v>
       </c>
@@ -3304,7 +3622,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A106">
         <v>105</v>
       </c>
@@ -3321,7 +3639,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A107">
         <v>106</v>
       </c>
@@ -3338,7 +3656,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A108">
         <v>107</v>
       </c>
@@ -3355,7 +3673,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A109">
         <v>108</v>
       </c>
@@ -3372,7 +3690,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A110">
         <v>109</v>
       </c>
@@ -3389,7 +3707,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A111">
         <v>110</v>
       </c>
@@ -3406,7 +3724,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A112">
         <v>111</v>
       </c>
@@ -4869,6 +5187,9 @@
       </c>
     </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="H5:I28">
+    <sortCondition descending="1" ref="I5:I28"/>
+  </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>